<commit_message>
Track identity balance as the library grows
Splits the Identities counter into Integration / Discovery / Total /
Share so imbalance is visible as concepts are added, and warns on a
Discovery concept with no identity tag.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XFMAvXhVPs5p7gV2TkcYmn
</commit_message>
<xml_diff>
--- a/content/praxis-concept-library.xlsx
+++ b/content/praxis-concept-library.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3575" uniqueCount="1573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3578" uniqueCount="1574">
   <si>
     <t xml:space="preserve">Status</t>
   </si>
@@ -4584,7 +4584,10 @@
     <t xml:space="preserve">Folds in</t>
   </si>
   <si>
-    <t xml:space="preserve">Concepts tagged</t>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of library</t>
   </si>
   <si>
     <t xml:space="preserve">I am a critical thinker</t>
@@ -4635,7 +4638,8 @@
     <t xml:space="preserve">Stops self-sabotage</t>
   </si>
   <si>
-    <t xml:space="preserve">Nothing is tagged yet — all 300 concepts need an Identity Tag pass, and that is Phase 1 work. Until a concept carries a tag it can never be surfaced by a goal or weight the wheel.
+    <t xml:space="preserve">Integration concepts are the expensive ones — they need a Praxis Exercise written. Discovery concepts are roughly half the work. Watch the Share column as the library grows: if one identity drifts far above the others, users who pick it get a weighted wheel full of material while users on a thin identity get very little. A first slice is a COUNT you choose (say 15 concepts), not a whole identity.
+Nothing is tagged yet — all 300 concepts need an Identity Tag pass, and that is Phase 1 work. Until a concept carries a tag it can never be surfaced by a goal or weight the wheel.
 Cut deliberately: 'high self confidence &amp; self worth' names a feeling, not a practice. There is no instance of it a user can log. Test for anything added: can a user point to a specific thing they did, on a specific day, that counts as evidence? Spelling must match the Vocabulary sheet exactly — matching is literal and a typo fails silently.</t>
   </si>
   <si>
@@ -4763,9 +4767,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -4913,7 +4918,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4944,6 +4949,14 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -21992,13 +22005,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22012,7 +22026,16 @@
         <v>1514</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>1515</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1516</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22020,14 +22043,26 @@
         <v>30</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>1517</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A2&amp;"*")</f>
+        <v>1518</v>
+      </c>
+      <c r="D2" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A2&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>101</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A2&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>45</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <f aca="false">D2+E2</f>
         <v>146</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <f aca="false">IFERROR($F2/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.486666666666667</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22035,14 +22070,26 @@
         <v>302</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1519</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A3&amp;"*")</f>
+        <v>1520</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A3&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>49</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A3&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>4</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <f aca="false">D3+E3</f>
         <v>53</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <f aca="false">IFERROR($F3/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.176666666666667</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22050,14 +22097,26 @@
         <v>556</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>1521</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A4&amp;"*")</f>
+        <v>1522</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A4&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>25</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A4&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>7</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <f aca="false">D4+E4</f>
         <v>32</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <f aca="false">IFERROR($F4/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.106666666666667</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22065,14 +22124,26 @@
         <v>322</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1523</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A5&amp;"*")</f>
+        <v>1524</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A5&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>34</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A5&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>13</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <f aca="false">D5+E5</f>
         <v>47</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <f aca="false">IFERROR($F5/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.156666666666667</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22080,14 +22151,26 @@
         <v>374</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>1525</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A6&amp;"*")</f>
+        <v>1526</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A6&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>41</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A6&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>21</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <f aca="false">D6+E6</f>
         <v>62</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <f aca="false">IFERROR($F6/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.206666666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22095,14 +22178,26 @@
         <v>527</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1527</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A7&amp;"*")</f>
+        <v>1528</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A7&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>18</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A7&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>20</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <f aca="false">D7+E7</f>
         <v>38</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <f aca="false">IFERROR($F7/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.126666666666667</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22110,14 +22205,26 @@
         <v>1018</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>1529</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A8&amp;"*")</f>
+        <v>1530</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A8&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>20</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A8&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>11</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <f aca="false">D8+E8</f>
         <v>31</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <f aca="false">IFERROR($F8/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.103333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22125,51 +22232,96 @@
         <v>233</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1531</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"*"&amp;$A9&amp;"*")</f>
+        <v>1532</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A9&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
+        <v>37</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A9&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
+        <v>45</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <f aca="false">D9+E9</f>
         <v>82</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <f aca="false">IFERROR($F9/COUNTA(Concepts!$C$2:$C$400),0)</f>
+        <v>0.273333333333333</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A11:D15"/>
+    <mergeCell ref="A11:G17"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -22194,255 +22346,255 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
-        <v>1533</v>
+      <c r="A1" s="10" t="s">
+        <v>1534</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>1534</v>
+      <c r="A2" s="11" t="s">
+        <v>1535</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>1535</v>
-      </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
+      <c r="A4" s="12" t="s">
+        <v>1536</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>1536</v>
-      </c>
-      <c r="B5" s="13" t="n">
+      <c r="A5" s="14" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B5" s="15" t="n">
         <f aca="false">COUNTA(Concepts!$C$2:$C$400)</f>
         <v>300</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="14" t="s">
         <v>1220</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="15" t="n">
         <f aca="false">COUNTIF(Concepts!$A$2:$A$400,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>1537</v>
-      </c>
-      <c r="B7" s="13" t="n">
+      <c r="A7" s="14" t="s">
+        <v>1538</v>
+      </c>
+      <c r="B7" s="15" t="n">
         <f aca="false">COUNTIF(Concepts!$A$2:$A$400,"Drafted")+COUNTIF(Concepts!$A$2:$A$400,"In review")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>1538</v>
-      </c>
-      <c r="B8" s="13" t="n">
+      <c r="A8" s="14" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B8" s="15" t="n">
         <f aca="false">COUNTIF(Concepts!$A$2:$A$400,"Stub")</f>
         <v>300</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>1539</v>
-      </c>
-      <c r="B9" s="13" t="n">
+      <c r="A9" s="14" t="s">
+        <v>1540</v>
+      </c>
+      <c r="B9" s="15" t="n">
         <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"?*")</f>
         <v>300</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>1540</v>
-      </c>
-      <c r="B10" s="13" t="n">
+      <c r="A10" s="14" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B10" s="15" t="n">
         <f aca="false">COUNTIF(Concepts!$D$2:$D$400,"?*")</f>
         <v>300</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>1541</v>
-      </c>
-      <c r="B11" s="13" t="n">
+      <c r="A11" s="14" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B11" s="15" t="n">
         <f aca="false">COUNTA(Books!$B$2:$B$300)</f>
         <v>133</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>1542</v>
-      </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
+      <c r="A13" s="12" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
-        <v>1543</v>
-      </c>
-      <c r="B14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>1544</v>
       </c>
+      <c r="B14" s="17" t="s">
+        <v>1545</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
-        <v>1545</v>
-      </c>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>1546</v>
       </c>
+      <c r="B15" s="17" t="s">
+        <v>1547</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
-        <v>1547</v>
-      </c>
-      <c r="B16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>1548</v>
       </c>
+      <c r="B16" s="17" t="s">
+        <v>1549</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>1549</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
+      <c r="A18" s="12" t="s">
+        <v>1550</v>
+      </c>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>1550</v>
-      </c>
-      <c r="B19" s="15" t="s">
+      <c r="A19" s="16" t="s">
         <v>1551</v>
       </c>
+      <c r="B19" s="17" t="s">
+        <v>1552</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
-        <v>1552</v>
-      </c>
-      <c r="B20" s="15" t="s">
+      <c r="A20" s="16" t="s">
         <v>1553</v>
       </c>
+      <c r="B20" s="17" t="s">
+        <v>1554</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>1554</v>
-      </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
+      <c r="A22" s="12" t="s">
+        <v>1555</v>
+      </c>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="15" t="s">
-        <v>1555</v>
+      <c r="B23" s="17" t="s">
+        <v>1556</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>1556</v>
+      <c r="B24" s="17" t="s">
+        <v>1557</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
-        <v>1557</v>
-      </c>
-      <c r="B25" s="15" t="s">
+      <c r="A25" s="16" t="s">
         <v>1558</v>
       </c>
+      <c r="B25" s="17" t="s">
+        <v>1559</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="15" t="s">
-        <v>1559</v>
+      <c r="B26" s="17" t="s">
+        <v>1560</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>1560</v>
+      <c r="B27" s="17" t="s">
+        <v>1561</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="15" t="s">
-        <v>1561</v>
+      <c r="B28" s="17" t="s">
+        <v>1562</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="15" t="s">
-        <v>1562</v>
+      <c r="B29" s="17" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>1563</v>
+      <c r="B30" s="17" t="s">
+        <v>1564</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>1564</v>
+      <c r="B31" s="17" t="s">
+        <v>1565</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="15" t="s">
-        <v>1565</v>
+      <c r="B32" s="17" t="s">
+        <v>1566</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
-        <v>1566</v>
-      </c>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
+      <c r="A34" s="12" t="s">
+        <v>1567</v>
+      </c>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="s">
-        <v>1567</v>
-      </c>
-      <c r="B35" s="15" t="s">
+      <c r="A35" s="16" t="s">
         <v>1568</v>
       </c>
+      <c r="B35" s="17" t="s">
+        <v>1569</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
-        <v>1569</v>
-      </c>
-      <c r="B36" s="15" t="s">
+      <c r="A36" s="16" t="s">
         <v>1570</v>
       </c>
+      <c r="B36" s="17" t="s">
+        <v>1571</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="s">
-        <v>1571</v>
-      </c>
-      <c r="B37" s="15" t="s">
+      <c r="A37" s="16" t="s">
         <v>1572</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>1573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace gap throughout the reader-facing copy
Ten uses across the page and the concept content, each rewritten to fit
its own sentence rather than swapped for one word everywhere: blind
spot, pause, difference, steps, missing pieces, weak points, what is
missing. The Curse of Knowledge exercise is now Name What You Skipped.

CSS gap properties are layout and are untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XFMAvXhVPs5p7gV2TkcYmn
</commit_message>
<xml_diff>
--- a/content/praxis-concept-library.xlsx
+++ b/content/praxis-concept-library.xlsx
@@ -1927,7 +1927,7 @@
     <t xml:space="preserve">REFLECTIVE LISTENING. That is one technique inside this practice, where you say back what you understood. Active listening is the wider posture of attending to meaning first, which can be shown in many ways besides reflecting.</t>
   </si>
   <si>
-    <t xml:space="preserve">Priya's colleague starts describing a problem with the schedule. Twenty seconds in, Priya has the answer and is waiting for a gap to say it. She delivers a good solution. Her colleague thanks her, and does not mention the part he had not got to yet, which was the actual difficulty.</t>
+    <t xml:space="preserve">Priya's colleague starts describing a problem with the schedule. Twenty seconds in, Priya has the answer and is waiting for a pause to say it. She delivers a good solution. Her colleague thanks her, and does not mention the part he had not got to yet, which was the actual difficulty.</t>
   </si>
   <si>
     <t xml:space="preserve">THE NO REPLY MINUTE
@@ -1980,7 +1980,7 @@
 1. Pick a conversation where you and the other person keep missing each other.
 2. Before responding, say: so what I am hearing is, and then put their point in your own words.
 3. Ask whether that is right.
-4. Write down what they corrected. That gap is what you had been answering.
+4. Write down what they corrected. That difference is what you had been answering.
 COMMITMENT (if then):
 "When a conversation feels like it is going in circles, I will restate their point in my own words and ask if I have it."</t>
   </si>
@@ -2213,13 +2213,13 @@
     <t xml:space="preserve">Once you know something, you cannot imagine not knowing it.</t>
   </si>
   <si>
-    <t xml:space="preserve">A bias in which knowing something makes it very hard to model the mind of someone who does not. It shows up whenever an expert explains their field: the gaps they skip are invisible to them, because the knowledge that fills those gaps is already in place. Demonstrated memorably in Elizabeth Newton's tapping study, where tappers wildly overestimated how often listeners would recognise the tune.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">you acquire knowledge -&gt; it becomes automatic -&gt; it stops feeling like knowledge -&gt; you leave it out -&gt; the listener loses the thread where you did not notice a gap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"It means experts are bad communicators." Expertise is not the problem; the invisibility of one's own knowledge is. A novice explaining something they half-know is often clearer, not because they know more but because the gaps are still visible to them.</t>
+    <t xml:space="preserve">A bias in which knowing something makes it very hard to model the mind of someone who does not. It shows up whenever an expert explains their field: the steps they skip are invisible to them, because the knowledge that fills them is already in place. Demonstrated memorably in Elizabeth Newton's tapping study, where tappers wildly overestimated how often listeners would recognise the tune.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">you acquire knowledge -&gt; it becomes automatic -&gt; it stops feeling like knowledge -&gt; you leave it out -&gt; the listener loses the thread where you skipped something without noticing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"It means experts are bad communicators." Expertise is not the problem; the invisibility of one's own knowledge is. A novice explaining something they half-know is often clearer, not because they know more but because the missing pieces are still visible to them.</t>
   </si>
   <si>
     <t xml:space="preserve">ILLUSION OF EXPLANATORY DEPTH. That one is about overestimating how well you understand something yourself. This one is about underestimating how much other people need told. One is a misjudgement of your own knowledge, the other a misjudgement of theirs.</t>
@@ -2228,7 +2228,7 @@
     <t xml:space="preserve">A consultant presents to a new client and uses four abbreviations in the first two minutes without expanding any of them. The room nods along. Afterwards almost no one can describe what was proposed, and the consultant concludes that the client was not paying attention.</t>
   </si>
   <si>
-    <t xml:space="preserve">NAME THE GAP
+    <t xml:space="preserve">NAME WHAT YOU SKIPPED
 1. Take something you are about to explain or publish.
 2. Underline every term that would need explaining to someone outside your field.
 3. For each, ask: did I actually explain it, or assume it?
@@ -3072,11 +3072,11 @@
     <t xml:space="preserve">Explain it simply, and the parts you cannot explain are what you do not know.</t>
   </si>
   <si>
-    <t xml:space="preserve">A study method in which you write an explanation of a topic as though to someone with no background, find the points where the explanation fails or retreats into jargon, go back to the source for those points specifically, and repeat. Its value is diagnostic: it locates gaps rather than filling them.</t>
+    <t xml:space="preserve">A study method in which you write an explanation of a topic as though to someone with no background, find the points where the explanation fails or retreats into jargon, go back to the source for those points specifically, and repeat. Its value is diagnostic: it locates what is missing rather than filling it.</t>
   </si>
   <si>
     <t xml:space="preserve">you reread material -&gt; it feels familiar -&gt; familiarity is mistaken for understanding
-you explain it plainly -&gt; the gaps refuse to be explained -&gt; you now know exactly what to go back for</t>
+you explain it plainly -&gt; the weak points refuse to be explained -&gt; you now know exactly what to go back for</t>
   </si>
   <si>
     <t xml:space="preserve">"It is about making things simple." Simplicity is the test, not the goal. The output is not meant to be a simplified explanation you keep. The output is the list of places where you could not manage it, and those are the only part worth acting on.</t>

</xml_diff>

<commit_message>
Rename Systems literate to Sees power structures and narrow it
Systems literate was a library word rather than something a person
would say about themselves. It also covered two unrelated things.

Of the 61 concepts only 33 were genuinely about power or strategy. The
other 28 were institutions, economics and collective behaviour, which
is a different subject: Tragedy of the Commons, Goodhart's Law, Network
Effects, Comparative Advantage, Catallaxy, the Malthusian Trap. Those
move to Clear thinker, taking it to 125.

Sees power structures now holds game theory, negotiation, the Galbraith
and Russell power types, Machiavelli, and how people stage themselves
in front of others. The claim is: I can see the game being played.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XFMAvXhVPs5p7gV2TkcYmn
</commit_message>
<xml_diff>
--- a/content/praxis-concept-library.xlsx
+++ b/content/praxis-concept-library.xlsx
@@ -2667,7 +2667,7 @@
     <t xml:space="preserve">Sociology / Social Exchange Theory</t>
   </si>
   <si>
-    <t xml:space="preserve">Manipulation proof; Systems literate</t>
+    <t xml:space="preserve">Manipulation proof; Sees power structures</t>
   </si>
   <si>
     <t xml:space="preserve">07.03</t>
@@ -2691,7 +2691,7 @@
     <t xml:space="preserve">Military Strategy</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate; Disciplined</t>
+    <t xml:space="preserve">Sees power structures; Disciplined</t>
   </si>
   <si>
     <t xml:space="preserve">BK056; BK082</t>
@@ -2706,7 +2706,7 @@
     <t xml:space="preserve">Military / Competitive Strategy</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate</t>
+    <t xml:space="preserve">Sees power structures</t>
   </si>
   <si>
     <t xml:space="preserve">BK082; BK084</t>
@@ -2784,7 +2784,7 @@
     <t xml:space="preserve">Negotiation Theory</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate; Manipulation proof</t>
+    <t xml:space="preserve">Sees power structures; Manipulation proof</t>
   </si>
   <si>
     <t xml:space="preserve">07.12</t>
@@ -2881,7 +2881,7 @@
     <t xml:space="preserve">Repeated Games</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate; High integrity</t>
+    <t xml:space="preserve">Sees power structures; High integrity</t>
   </si>
   <si>
     <t xml:space="preserve">07.18</t>
@@ -2908,7 +2908,7 @@
     <t xml:space="preserve">Game Theory / Coordination</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate; Clear communicator</t>
+    <t xml:space="preserve">Sees power structures; Clear communicator</t>
   </si>
   <si>
     <t xml:space="preserve">BK118</t>
@@ -4513,7 +4513,7 @@
     <t xml:space="preserve">Microsociology</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate; Self-authoring</t>
+    <t xml:space="preserve">Sees power structures; Self-authoring</t>
   </si>
   <si>
     <t xml:space="preserve">BK062</t>
@@ -6394,7 +6394,7 @@
     <t xml:space="preserve">The Third Alternative</t>
   </si>
   <si>
-    <t xml:space="preserve">Clear communicator; Systems literate</t>
+    <t xml:space="preserve">Clear communicator; Sees power structures</t>
   </si>
   <si>
     <t xml:space="preserve">03.44</t>
@@ -6631,7 +6631,7 @@
     <t xml:space="preserve">Everyday Mind</t>
   </si>
   <si>
-    <t xml:space="preserve">Systems literate; Emotionally regulated</t>
+    <t xml:space="preserve">Sees power structures; Emotionally regulated</t>
   </si>
   <si>
     <t xml:space="preserve">BK084</t>
@@ -7941,10 +7941,10 @@
     <t xml:space="preserve">Weighs risk; resists the biases that distort choosing; knows what a number does and does not tell them</t>
   </si>
   <si>
-    <t xml:space="preserve">I see why things turn out as they do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reads incentives, institutions and power; understands why good people can produce bad outcomes</t>
+    <t xml:space="preserve">I can see the game being played</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Game theory, negotiation and strategy; the Galbraith and Russell power types; Machiavelli; how people stage themselves in front of others</t>
   </si>
   <si>
     <t xml:space="preserve">Clear thinker was split in three on 4 October. It had grown to 209 concepts, forty three per cent of the library, which meant a user choosing it got almost half of everything weighted toward them while a user on a thin identity got very little. Reasoning and logic stayed as Clear thinker. Decisions under uncertainty became Sound judgement. Incentives, institutions and power became Systems literate.
@@ -8234,7 +8234,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -8264,10 +8264,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -22432,7 +22428,7 @@
       <c r="S277" s="4"/>
       <c r="T277" s="4"/>
       <c r="U277" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V277" s="3"/>
       <c r="W277" s="3" t="s">
@@ -22667,7 +22663,7 @@
       <c r="S282" s="4"/>
       <c r="T282" s="4"/>
       <c r="U282" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V282" s="3"/>
       <c r="W282" s="3" t="s">
@@ -22714,7 +22710,7 @@
       <c r="S283" s="4"/>
       <c r="T283" s="4"/>
       <c r="U283" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V283" s="3"/>
       <c r="W283" s="3" t="s">
@@ -22761,7 +22757,7 @@
       <c r="S284" s="4"/>
       <c r="T284" s="4"/>
       <c r="U284" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V284" s="3"/>
       <c r="W284" s="3" t="s">
@@ -22808,7 +22804,7 @@
       <c r="S285" s="4"/>
       <c r="T285" s="4"/>
       <c r="U285" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V285" s="3"/>
       <c r="W285" s="3" t="s">
@@ -22855,7 +22851,7 @@
       <c r="S286" s="4"/>
       <c r="T286" s="4"/>
       <c r="U286" s="4" t="s">
-        <v>905</v>
+        <v>75</v>
       </c>
       <c r="V286" s="3"/>
       <c r="W286" s="3" t="s">
@@ -22902,7 +22898,7 @@
       <c r="S287" s="4"/>
       <c r="T287" s="4"/>
       <c r="U287" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V287" s="3"/>
       <c r="W287" s="3" t="s">
@@ -22949,7 +22945,7 @@
       <c r="S288" s="4"/>
       <c r="T288" s="4"/>
       <c r="U288" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V288" s="3"/>
       <c r="W288" s="3" t="s">
@@ -22996,7 +22992,7 @@
       <c r="S289" s="4"/>
       <c r="T289" s="4"/>
       <c r="U289" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V289" s="3"/>
       <c r="W289" s="3" t="s">
@@ -23043,7 +23039,7 @@
       <c r="S290" s="4"/>
       <c r="T290" s="4"/>
       <c r="U290" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V290" s="3"/>
       <c r="W290" s="3" t="s">
@@ -23090,7 +23086,7 @@
       <c r="S291" s="4"/>
       <c r="T291" s="4"/>
       <c r="U291" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V291" s="3"/>
       <c r="W291" s="3" t="s">
@@ -23184,7 +23180,7 @@
       <c r="S293" s="4"/>
       <c r="T293" s="4"/>
       <c r="U293" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V293" s="3"/>
       <c r="W293" s="3" t="s">
@@ -23231,7 +23227,7 @@
       <c r="S294" s="4"/>
       <c r="T294" s="4"/>
       <c r="U294" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V294" s="3"/>
       <c r="W294" s="3" t="s">
@@ -23278,7 +23274,7 @@
       <c r="S295" s="4"/>
       <c r="T295" s="4"/>
       <c r="U295" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V295" s="3"/>
       <c r="W295" s="3" t="s">
@@ -23325,7 +23321,7 @@
       <c r="S296" s="4"/>
       <c r="T296" s="4"/>
       <c r="U296" s="4" t="s">
-        <v>844</v>
+        <v>58</v>
       </c>
       <c r="V296" s="3"/>
       <c r="W296" s="3" t="s">
@@ -23372,7 +23368,7 @@
       <c r="S297" s="4"/>
       <c r="T297" s="4"/>
       <c r="U297" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V297" s="3"/>
       <c r="W297" s="3" t="s">
@@ -23419,7 +23415,7 @@
       <c r="S298" s="4"/>
       <c r="T298" s="4"/>
       <c r="U298" s="4" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
       <c r="V298" s="3"/>
       <c r="W298" s="3" t="s">
@@ -23513,7 +23509,7 @@
       <c r="S300" s="4"/>
       <c r="T300" s="4"/>
       <c r="U300" s="4" t="s">
-        <v>875</v>
+        <v>92</v>
       </c>
       <c r="V300" s="3"/>
       <c r="W300" s="3" t="s">
@@ -27012,7 +27008,7 @@
       </c>
       <c r="N380" s="3"/>
       <c r="U380" s="3" t="s">
-        <v>875</v>
+        <v>92</v>
       </c>
     </row>
     <row r="381" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27039,7 +27035,7 @@
       </c>
       <c r="N381" s="3"/>
       <c r="U381" s="3" t="s">
-        <v>875</v>
+        <v>92</v>
       </c>
     </row>
     <row r="382" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27066,7 +27062,7 @@
       </c>
       <c r="N382" s="3"/>
       <c r="U382" s="3" t="s">
-        <v>914</v>
+        <v>124</v>
       </c>
     </row>
     <row r="383" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27093,7 +27089,7 @@
       </c>
       <c r="N383" s="3"/>
       <c r="U383" s="3" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
     </row>
     <row r="384" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27219,7 +27215,7 @@
       </c>
       <c r="N386" s="3"/>
       <c r="U386" s="3" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
     </row>
     <row r="387" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27246,7 +27242,7 @@
       </c>
       <c r="N387" s="3"/>
       <c r="U387" s="3" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
     </row>
     <row r="388" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27273,7 +27269,7 @@
       </c>
       <c r="N388" s="3"/>
       <c r="U388" s="3" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
     </row>
     <row r="389" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27300,7 +27296,7 @@
       </c>
       <c r="N389" s="3"/>
       <c r="U389" s="3" t="s">
-        <v>849</v>
+        <v>43</v>
       </c>
     </row>
     <row r="390" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27645,7 +27641,7 @@
         <v>295</v>
       </c>
       <c r="U401" s="3" t="s">
-        <v>875</v>
+        <v>92</v>
       </c>
       <c r="W401" s="3" t="s">
         <v>2014</v>
@@ -27964,7 +27960,7 @@
         <v>442</v>
       </c>
       <c r="U412" s="3" t="s">
-        <v>875</v>
+        <v>92</v>
       </c>
       <c r="W412" s="3" t="s">
         <v>231</v>
@@ -30345,7 +30341,7 @@
       <c r="B10" s="7" t="s">
         <v>1455</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>202</v>
       </c>
     </row>
@@ -30356,7 +30352,7 @@
       <c r="B11" s="7" t="s">
         <v>510</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>849</v>
       </c>
     </row>
@@ -30467,83 +30463,83 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9"/>
+      <c r="A32" s="8"/>
       <c r="B32" s="7" t="s">
         <v>612</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="9" t="s">
         <v>2206</v>
       </c>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
+      <c r="A35" s="9"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
+      <c r="A36" s="9"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -33257,7 +33253,7 @@
       <c r="F135" s="3" t="s">
         <v>2490</v>
       </c>
-      <c r="G135" s="11" t="n">
+      <c r="G135" s="10" t="n">
         <f aca="false">IF($A135="","",COUNTIF(Concepts!$V$2:$V$400,"*"&amp;$A135&amp;"*"))</f>
         <v>0</v>
       </c>
@@ -33278,7 +33274,7 @@
       <c r="E136" s="3" t="s">
         <v>2489</v>
       </c>
-      <c r="G136" s="11" t="n">
+      <c r="G136" s="10" t="n">
         <f aca="false">IF($A136="","",COUNTIF(Concepts!$W$2:$W$400,"*"&amp;$A136&amp;"*"))</f>
         <v>1</v>
       </c>
@@ -33299,7 +33295,7 @@
       <c r="E137" s="3" t="s">
         <v>2489</v>
       </c>
-      <c r="G137" s="11" t="n">
+      <c r="G137" s="10" t="n">
         <f aca="false">IF($A137="","",COUNTIF(Concepts!$W$2:$W$400,"*"&amp;$A137&amp;"*"))</f>
         <v>2</v>
       </c>
@@ -33320,7 +33316,7 @@
       <c r="E138" s="3" t="s">
         <v>2489</v>
       </c>
-      <c r="G138" s="11" t="n">
+      <c r="G138" s="10" t="n">
         <f aca="false">IF($A138="","",COUNTIF(Concepts!$W$2:$W$400,"*"&amp;$A138&amp;"*"))</f>
         <v>10</v>
       </c>
@@ -33341,7 +33337,7 @@
       <c r="E139" s="3" t="s">
         <v>2489</v>
       </c>
-      <c r="G139" s="11" t="n">
+      <c r="G139" s="10" t="n">
         <f aca="false">IF($A139="","",COUNTIF(Concepts!$W$2:$W$400,"*"&amp;$A139&amp;"*"))</f>
         <v>2</v>
       </c>
@@ -33362,7 +33358,7 @@
       <c r="E140" s="3" t="s">
         <v>2489</v>
       </c>
-      <c r="G140" s="11" t="n">
+      <c r="G140" s="10" t="n">
         <f aca="false">IF($A140="","",COUNTIF(Concepts!$W$2:$W$400,"*"&amp;$A140&amp;"*"))</f>
         <v>0</v>
       </c>
@@ -33370,33 +33366,33 @@
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="143" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C143" s="9" t="s">
+      <c r="C143" s="8" t="s">
         <v>2498</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C144" s="12"/>
-      <c r="D144" s="12"/>
-      <c r="E144" s="12"/>
-      <c r="F144" s="12"/>
-      <c r="G144" s="12"/>
-      <c r="H144" s="12"/>
+      <c r="C144" s="11"/>
+      <c r="D144" s="11"/>
+      <c r="E144" s="11"/>
+      <c r="F144" s="11"/>
+      <c r="G144" s="11"/>
+      <c r="H144" s="11"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C145" s="12"/>
-      <c r="D145" s="12"/>
-      <c r="E145" s="12"/>
-      <c r="F145" s="12"/>
-      <c r="G145" s="12"/>
-      <c r="H145" s="12"/>
+      <c r="C145" s="11"/>
+      <c r="D145" s="11"/>
+      <c r="E145" s="11"/>
+      <c r="F145" s="11"/>
+      <c r="G145" s="11"/>
+      <c r="H145" s="11"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C146" s="12"/>
-      <c r="D146" s="12"/>
-      <c r="E146" s="12"/>
-      <c r="F146" s="12"/>
-      <c r="G146" s="12"/>
-      <c r="H146" s="12"/>
+      <c r="C146" s="11"/>
+      <c r="D146" s="11"/>
+      <c r="E146" s="11"/>
+      <c r="F146" s="11"/>
+      <c r="G146" s="11"/>
+      <c r="H146" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H134"/>
@@ -33452,7 +33448,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -33461,25 +33457,25 @@
       <c r="C2" s="3" t="s">
         <v>2505</v>
       </c>
-      <c r="D2" s="14" t="n">
+      <c r="D2" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A2&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A2&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F2" s="14" t="n">
+      <c r="F2" s="13" t="n">
         <f aca="false">D2+E2</f>
         <v>0</v>
       </c>
-      <c r="G2" s="15" t="n">
+      <c r="G2" s="14" t="n">
         <f aca="false">IFERROR($F2/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>385</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -33488,25 +33484,25 @@
       <c r="C3" s="3" t="s">
         <v>2507</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A3&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A3&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="F3" s="13" t="n">
         <f aca="false">D3+E3</f>
         <v>0</v>
       </c>
-      <c r="G3" s="15" t="n">
+      <c r="G3" s="14" t="n">
         <f aca="false">IFERROR($F3/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="12" t="s">
         <v>690</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -33515,25 +33511,25 @@
       <c r="C4" s="3" t="s">
         <v>2509</v>
       </c>
-      <c r="D4" s="14" t="n">
+      <c r="D4" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A4&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A4&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="13" t="n">
         <f aca="false">D4+E4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="14" t="n">
         <f aca="false">IFERROR($F4/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
         <v>405</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -33542,25 +33538,25 @@
       <c r="C5" s="3" t="s">
         <v>2511</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A5&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A5&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="13" t="n">
         <f aca="false">D5+E5</f>
         <v>0</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="14" t="n">
         <f aca="false">IFERROR($F5/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="12" t="s">
         <v>458</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -33569,25 +33565,25 @@
       <c r="C6" s="3" t="s">
         <v>2513</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A6&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A6&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="13" t="n">
         <f aca="false">D6+E6</f>
         <v>0</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="14" t="n">
         <f aca="false">IFERROR($F6/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="12" t="s">
         <v>624</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -33596,25 +33592,25 @@
       <c r="C7" s="3" t="s">
         <v>2515</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A7&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A7&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="13" t="n">
         <f aca="false">D7+E7</f>
         <v>0</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="14" t="n">
         <f aca="false">IFERROR($F7/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="12" t="s">
         <v>1314</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -33623,25 +33619,25 @@
       <c r="C8" s="3" t="s">
         <v>2517</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A8&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A8&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="13" t="n">
         <f aca="false">D8+E8</f>
         <v>0</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="14" t="n">
         <f aca="false">IFERROR($F8/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="12" t="s">
         <v>304</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -33650,25 +33646,25 @@
       <c r="C9" s="3" t="s">
         <v>2519</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A9&amp;"*",Concepts!$D$2:$D$400,"Integration")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">COUNTIFS(Concepts!$S$2:$S$400,"*"&amp;$A9&amp;"*",Concepts!$D$2:$D$400,"Discovery")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="13" t="n">
         <f aca="false">D9+E9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="14" t="n">
         <f aca="false">IFERROR($F9/COUNTA(Concepts!$C$2:$C$400),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="12" t="s">
         <v>202</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -33689,13 +33685,13 @@
         <f aca="false">D10+E10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="15" t="n">
         <f aca="false">IFERROR($F10/COUNTA(Concepts!$C$2:$C$600),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="12" t="s">
         <v>849</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -33716,103 +33712,103 @@
         <f aca="false">D11+E11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="15" t="n">
         <f aca="false">IFERROR($F11/COUNTA(Concepts!$C$2:$C$600),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="9" t="s">
         <v>2524</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -33841,271 +33837,271 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>2525</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>2526</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>2527</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="20" t="s">
         <v>2528</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="10" t="n">
         <f aca="false">COUNTA(Concepts!$C$2:$C$400)</f>
         <v>399</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="10" t="n">
         <f aca="false">COUNTIF(Concepts!$A$2:$A$400,"Done")</f>
         <v>60</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="20" t="s">
         <v>2529</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">COUNTIF(Concepts!$A$2:$A$400,"Drafted")+COUNTIF(Concepts!$A$2:$A$400,"In review")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="20" t="s">
         <v>2530</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="10" t="n">
         <f aca="false">COUNTIF(Concepts!$A$2:$A$400,"Stub")</f>
         <v>339</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="20" t="s">
         <v>2531</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="10" t="n">
         <f aca="false">COUNTIF(Concepts!$S$2:$S$400,"?*")</f>
         <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="20" t="s">
         <v>2532</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="10" t="n">
         <f aca="false">COUNTIF(Concepts!$D$2:$D$400,"?*")</f>
         <v>399</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="20" t="s">
         <v>2533</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="10" t="n">
         <f aca="false">COUNTA(Books!$B$2:$B$300)</f>
         <v>138</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>2534</v>
       </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="21" t="s">
         <v>2535</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="22" t="s">
         <v>2536</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="21" t="s">
         <v>2537</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="22" t="s">
         <v>2538</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="21" t="s">
         <v>2539</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="22" t="s">
         <v>2540</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>2541</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="21" t="s">
         <v>2542</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="22" t="s">
         <v>2543</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="21" t="s">
         <v>2544</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="22" t="s">
         <v>2545</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="18" t="s">
         <v>2546</v>
       </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
     </row>
     <row r="23" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="22" t="s">
         <v>2547</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="22" t="s">
         <v>2548</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="22" t="s">
         <v>2549</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="23" t="s">
+      <c r="B26" s="22" t="s">
         <v>2550</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="21" t="s">
         <v>2551</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="22" t="s">
         <v>2552</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="22" t="s">
         <v>2553</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="23" t="s">
+      <c r="B29" s="22" t="s">
         <v>2554</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="23" t="s">
+      <c r="B30" s="22" t="s">
         <v>2555</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="22" t="s">
         <v>2556</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="22" t="s">
         <v>2557</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
+      <c r="A33" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="23" t="s">
+      <c r="B33" s="22" t="s">
         <v>2558</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="22" t="s">
         <v>2559</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="36" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="18" t="s">
         <v>2560</v>
       </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="21" t="s">
         <v>2561</v>
       </c>
-      <c r="B37" s="23" t="s">
+      <c r="B37" s="22" t="s">
         <v>2562</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="21" t="s">
         <v>2563</v>
       </c>
-      <c r="B38" s="23" t="s">
+      <c r="B38" s="22" t="s">
         <v>2564</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="22" t="s">
+      <c r="A39" s="21" t="s">
         <v>2565</v>
       </c>
-      <c r="B39" s="23" t="s">
+      <c r="B39" s="22" t="s">
         <v>2566</v>
       </c>
     </row>

</xml_diff>